<commit_message>
fix(uploads): standardize credentials to Test@123, auto-create unmatched students on group/thesis confirm, and clean faculty names in templates
</commit_message>
<xml_diff>
--- a/backend/excel-templates/New-Test-data/bachelor_external_users_test_data.xlsx
+++ b/backend/excel-templates/New-Test-data/bachelor_external_users_test_data.xlsx
@@ -435,19 +435,19 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>dr..lokendradhakal@ioe.edu.np</v>
+        <v>lokendra.dhakal@ioe.edu.np</v>
       </c>
       <c r="B3" t="str">
         <v>Test@123</v>
       </c>
       <c r="C3" t="str">
-        <v>Dr.</v>
+        <v>Lokendra</v>
       </c>
       <c r="D3" t="str">
-        <v>Lokendra Dhakal</v>
+        <v>Dhakal</v>
       </c>
       <c r="E3" t="str">
-        <v>Prof.</v>
+        <v>Prof. Dr.</v>
       </c>
     </row>
     <row r="4">
@@ -486,19 +486,19 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>prof..dr.manishaaryal@ioe.edu.np</v>
+        <v>manisha.aryal@ioe.edu.np</v>
       </c>
       <c r="B6" t="str">
         <v>Test@123</v>
       </c>
       <c r="C6" t="str">
-        <v>Prof.</v>
+        <v>Manisha</v>
       </c>
       <c r="D6" t="str">
-        <v>Dr. Manisha Aryal</v>
+        <v>Aryal</v>
       </c>
       <c r="E6" t="str">
-        <v>Assoc.</v>
+        <v>Assoc. Prof. Dr.</v>
       </c>
     </row>
     <row r="7">

</xml_diff>